<commit_message>
fix: remove unverified ISO main-body clause citations; validator now rejects them
17 clause-number references across 15 rows could not be verified against a
licensed copy. Rows now name the main-body topic without a number; Annex A
controls are the citation unit. Outputs rebuilt.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UyvLFEt1y6TF3PhdFdmV6p
</commit_message>
<xml_diff>
--- a/crosswalk/crosswalk.xlsx
+++ b/crosswalk/crosswalk.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>cl. 6.1.2 AI risk assessment; cl. 6.1.3 AI risk treatment; cl. 8.2-8.3 operational assessment/treatment; A.6.1.2 objectives for responsible development; A.6.1.3 processes for responsible design and development. Intent: a repeatable AI-risk process with treatment and residual-risk acceptance.</t>
+          <t>main-body AI risk assessment and risk treatment requirements; A.6.1.2 objectives for responsible development; A.6.1.3 processes for responsible design and development. Intent: a repeatable AI-risk process with treatment and residual-risk acceptance.</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>cl. 6.1.2-6.1.3 (information-security risk assessment/treatment) - covers the security slice only.</t>
+          <t>main-body information-security risk assessment and treatment requirements - covers the security slice only.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>A.6.2.4 AI system verification and validation; A.6.2.2 requirements and specification; cl. 8.1 operational planning. Intent: define and run V&amp;V against stated criteria.</t>
+          <t>A.6.2.4 AI system verification and validation; A.6.2.2 requirements and specification; main-body operational planning and control requirement. Intent: define and run V&amp;V against stated criteria.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>A.6.2.7 AI system technical documentation; A.6.2.3 Documentation of design and development; cl. 7.5 Documented information. Intent: maintain system-level documentation.</t>
+          <t>A.6.2.7 AI system technical documentation; A.6.2.3 Documentation of design and development; main-body documented-information requirement. Intent: maintain system-level documentation.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>A.4.5 System and computing resources; cl. 6.1.2 AI risk assessment. Intent: resourcing and risk assessment - no AI-specific security control exists in Annex A.</t>
+          <t>A.4.5 System and computing resources; main-body AI risk assessment requirement. Intent: resourcing and risk assessment - no AI-specific security control exists in Annex A.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>cl. 4-10 (whole AI management system); cl. 5.2 AI policy; cl. 7.5 documented information; A.2.2 AI policy; A.3.2 roles; A.6.2.2-A.6.2.8 AI system life-cycle controls; A.10.3 suppliers. Intent: a certified management system around AI development and use.</t>
+          <t>main-body requirements of the AI management system as a whole (policy, documented information and the rest); A.2.2 AI policy; A.3.2 roles; A.6.2.2-A.6.2.8 AI system life-cycle controls; A.10.3 suppliers. Intent: a certified management system around AI development and use.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>cl. 4-10 as the parallel ISMS (shared Annex SL structure) - supports integrated management-system operation.</t>
+          <t>main-body requirements of the parallel ISMS (same management-system structure) - supports integrated management-system operation.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>cl. 9.2 Internal audit; cl. 9.3 Management review. Intent: the organisation audits its own management system.</t>
+          <t>main-body internal audit and management review requirements (no Annex A control applies). Intent: the organisation audits its own management system.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>cl. 10.2 Nonconformity and corrective action; A.8.4 Communication of incidents; A.6.2.6 Operation and monitoring. Intent: fix and learn from nonconformities and incidents.</t>
+          <t>main-body nonconformity and corrective-action requirement; A.8.4 Communication of incidents; A.6.2.6 Operation and monitoring. Intent: fix and learn from nonconformities and incidents.</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>A.6.2.6 AI system operation and monitoring; cl. 9.1 Monitoring, measurement, analysis and evaluation; cl. 10.1 Continual improvement. Intent: monitor operation and improve.</t>
+          <t>A.6.2.6 AI system operation and monitoring; main-body monitoring/measurement and continual-improvement requirements. Intent: monitor operation and improve.</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>A.8.4 Communication of incidents; A.8.3 External reporting; cl. 10.2. Intent: communicate incidents to the right parties.</t>
+          <t>A.8.4 Communication of incidents; A.8.3 External reporting; main-body corrective-action requirement. Intent: communicate incidents to the right parties.</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>cl. 7.2 Competence; cl. 7.3 Awareness; A.4.6 Human resources; A.3.2 AI roles and responsibilities. Intent: people doing AI work are competent and aware.</t>
+          <t>main-body competence and awareness requirements; A.4.6 Human resources; A.3.2 AI roles and responsibilities. Intent: people doing AI work are competent and aware.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>cl. 7.2 Competence; cl. 7.3 Awareness; A.9.2 Processes for responsible use of AI systems; A.4.6 Human resources.</t>
+          <t>main-body competence and awareness requirements; A.9.2 Processes for responsible use of AI systems; A.4.6 Human resources.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>A.3.2 AI roles and responsibilities; A.4.6 Human resources; A.9.2; cl. 7.2 Competence. Intent: named, competent, resourced people.</t>
+          <t>A.3.2 AI roles and responsibilities; A.4.6 Human resources; A.9.2; main-body competence requirement. Intent: named, competent, resourced people.</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>A.5.2 AI system impact assessment process; A.5.3 Documentation of impact assessments; A.5.4 Impact on individuals or groups; cl. 6.1.4 / 8.4 AI system impact assessment. Intent: assess and document effects on individuals, groups and society.</t>
+          <t>A.5.2 AI system impact assessment process; A.5.3 Documentation of impact assessments; A.5.4 Impact on individuals or groups; main-body AI system impact assessment requirement. Intent: assess and document effects on individuals, groups and society.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>cl. 6.1.2 AI risk assessment; cl. 6.1.4 AI system impact assessment; A.5.5 Assessing societal impacts of AI systems. Intent: assess societal-level impacts.</t>
+          <t>main-body AI risk assessment and AI system impact assessment requirements; A.5.5 Assessing societal impacts of AI systems. Intent: assess societal-level impacts.</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>A.8.4 Communication of incidents; A.8.3 External reporting; cl. 10.2. Intent: tell the right parties about incidents.</t>
+          <t>A.8.4 Communication of incidents; A.8.3 External reporting; main-body corrective-action requirement. Intent: tell the right parties about incidents.</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">

</xml_diff>